<commit_message>
Fix fee calculations and add Windows build
</commit_message>
<xml_diff>
--- a/master/aliases_to_review.xlsx
+++ b/master/aliases_to_review.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="UnknownNames" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UnknownNames'!$A$1:$D$10</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -29,15 +31,25 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +57,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -134,6 +141,61 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SalaryCalc</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C7" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C9" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+    <comment ref="C10" authorId="0" shapeId="0">
+      <text>
+        <t>กรอกข้อมูลช่องนี้ก่อนนำไปใช้</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -425,8 +487,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -458,10 +526,10 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ทีม รพ. สมุทรสาคร</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Chatcharin Suksom</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
@@ -476,10 +544,10 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ทีม รพ.ราชธานี หนองแค</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Kasidate Dumnoo</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
@@ -494,10 +562,10 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ทีม รพ.ราชธานี อยุธยา</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Nattawan Chettanapiwat</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
@@ -512,17 +580,109 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Sirinya Phuphiewkam</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monitor Tech</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sirinya phuphiewkam</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Monitor Tech</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ทีม รพ. สมุทรสาคร</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Monitor Tech</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ทีม รพ.ราชธานี หนองแค</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Monitor Tech</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ทีม รพ.ราชธานี อยุธยา</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Monitor Tech</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>ทีม รพ.ราชธานี โรจนะ</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
         <is>
           <t>กรอก emp_code ให้ตรงกับพนักงาน แล้วนำข้อมูลนี้ไปเพิ่มใน aliases.xlsx</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>